<commit_message>
updated excel add information in add student such as address, age, emergency contact change text to icon
</commit_message>
<xml_diff>
--- a/project/students.xlsx
+++ b/project/students.xlsx
@@ -17,13 +17,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -46,8 +49,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,36 +419,74 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:K1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="40" customWidth="1" min="7" max="7"/>
+    <col width="28" customWidth="1" min="8" max="8"/>
+    <col width="32" customWidth="1" min="9" max="9"/>
+    <col width="26" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Student ID</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Name</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Course</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Year</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Age</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Contact Number</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Address</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Emergency Contact Name</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Emergency Contact Relationship</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Emergency Contact Number</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Status</t>
         </is>

</xml_diff>

<commit_message>
updated excel to be fitted their details/information adjust logo in dashboard remove dialog when logging in change password admin to PUPadmin2026!
</commit_message>
<xml_diff>
--- a/project/students.xlsx
+++ b/project/students.xlsx
@@ -9,7 +9,9 @@
   <sheets>
     <sheet name="Students" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Students'!$A$1:$K$1</definedName>
+  </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -27,14 +29,20 @@
     </font>
     <font>
       <b val="1"/>
+      <color rgb="0012313A"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00DFF7FB"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -51,8 +59,8 @@
   </cellStyleXfs>
   <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -424,18 +432,18 @@
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
     <col width="28" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="58" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
     <col width="8" customWidth="1" min="5" max="5"/>
     <col width="18" customWidth="1" min="6" max="6"/>
-    <col width="40" customWidth="1" min="7" max="7"/>
+    <col width="38" customWidth="1" min="7" max="7"/>
     <col width="28" customWidth="1" min="8" max="8"/>
-    <col width="32" customWidth="1" min="9" max="9"/>
-    <col width="26" customWidth="1" min="10" max="10"/>
+    <col width="34" customWidth="1" min="9" max="9"/>
+    <col width="28" customWidth="1" min="10" max="10"/>
     <col width="14" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="32" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Student ID</t>
@@ -493,6 +501,7 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:K1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
added gender in add student form updated excel add a gender remove in gender prefer not to say adjust logo
</commit_message>
<xml_diff>
--- a/project/students.xlsx
+++ b/project/students.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Students" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Students'!$A$1:$K$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Students'!$A$1:$L$1</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K1"/>
+  <dimension ref="A1:L1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -435,12 +435,13 @@
     <col width="58" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="8" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
-    <col width="38" customWidth="1" min="7" max="7"/>
-    <col width="28" customWidth="1" min="8" max="8"/>
-    <col width="34" customWidth="1" min="9" max="9"/>
-    <col width="28" customWidth="1" min="10" max="10"/>
-    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="38" customWidth="1" min="8" max="8"/>
+    <col width="28" customWidth="1" min="9" max="9"/>
+    <col width="34" customWidth="1" min="10" max="10"/>
+    <col width="28" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -471,37 +472,42 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
+          <t>Gender</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
           <t>Contact Number</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Address</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Emergency Contact Name</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Emergency Contact Relationship</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Emergency Contact Number</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K1"/>
+  <autoFilter ref="A1:L1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>